<commit_message>
Enter quencher redox potentials by hand instead of extracting them from the CVs
The voltammograms stay as raw exports. Potentials now live in two hand-edited
tables, quencher_redox_measured.csv (25 quenchers, CV) and
quencher_redox_literature.csv (23 quenchers, DOI or estimated), filled with
the values in use; quencher_redox_potentials.py joins them into
quencher_redox_potentials.csv, which is unchanged. The CV analysis script and
its two output tables are removed.
</commit_message>
<xml_diff>
--- a/data/experimental_data_processed/quencher_properties_exp.xlsx
+++ b/data/experimental_data_processed/quencher_properties_exp.xlsx
@@ -5966,7 +5966,7 @@
       <c r="C11" s="15" t="inlineStr"/>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>For a measured voltammogram, the value read (onset, half-wave, or no wave inside the window); otherwise the note from the literature file.</t>
+          <t>Free-text note from quencher_redox_measured.csv or quencher_redox_literature.csv.</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -6548,7 +6548,7 @@
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>One row per quencher. The potentials are read from the voltammogram for the 19</t>
+          <t>One row per quencher. The potentials are read by hand from the voltammograms or</t>
         </is>
       </c>
       <c r="B34" s="15" t="n"/>
@@ -6559,7 +6559,7 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>quenchers that have one, and taken from the literature for the others; both are in</t>
+          <t>taken from the literature, and entered in quencher_redox_measured.csv or</t>
         </is>
       </c>
       <c r="B35" s="15" t="n"/>
@@ -6570,7 +6570,7 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>experimental_data_raw/quencher_cyclic_voltammetry/.</t>
+          <t>quencher_redox_literature.csv in experimental_data_raw/quencher_cyclic_voltammetry/.</t>
         </is>
       </c>
       <c r="B36" s="15" t="n"/>

</xml_diff>

<commit_message>
Update quencher redox potentials from the manual reading
Revised measured and literature potentials, window-edge limits for the
missing channels, Q1 and Q16 moved to the literature table, and the
voltammograms moved to measured data/. exp_dataset_ent rebuilt: 939 pairs,
378 quenching.
</commit_message>
<xml_diff>
--- a/data/experimental_data_processed/quencher_properties_exp.xlsx
+++ b/data/experimental_data_processed/quencher_properties_exp.xlsx
@@ -766,14 +766,10 @@
       </c>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>measured by PPR; voltammogram not in the data</t>
-        </is>
-      </c>
+          <t>https://doi.org/10.1038/s41929-026-01566-z</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="n"/>
       <c r="M3" s="13" t="n">
         <v>0.0038773</v>
       </c>
@@ -962,8 +958,14 @@
           <t>CC1=C(C(=CC=C1)C)[N+](=O)[O-]</t>
         </is>
       </c>
-      <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="n"/>
+      <c r="F5" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
       <c r="H5" s="13" t="n">
         <v>-1.407</v>
       </c>
@@ -975,7 +977,7 @@
       </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
-          <t>converted from Fc/Fc+ to SCE</t>
+          <t>E_Red: converted from Fc/Fc+ to SCE; E_Ox: edge of the window</t>
         </is>
       </c>
       <c r="M5" s="13" t="n">
@@ -1166,8 +1168,14 @@
           <t>C12=NC=CN=C1C=CC=C2</t>
         </is>
       </c>
-      <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
+      <c r="F7" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
       <c r="H7" s="13" t="n">
         <v>-1.8</v>
       </c>
@@ -1177,7 +1185,11 @@
           <t>https://doi.org/10.1039/j19680000381</t>
         </is>
       </c>
-      <c r="K7" s="13" t="n"/>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>E_Ox: edge of the window</t>
+        </is>
+      </c>
       <c r="M7" s="13" t="n">
         <v>0.0226936</v>
       </c>
@@ -1263,8 +1275,14 @@
           <t>C12=CN=CC=C1C=CC=C2</t>
         </is>
       </c>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="13" t="n"/>
+      <c r="F8" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
       <c r="H8" s="13" t="n">
         <v>-2.2</v>
       </c>
@@ -1274,7 +1292,11 @@
           <t>https://doi.org/10.1039/j19680000381</t>
         </is>
       </c>
-      <c r="K8" s="13" t="n"/>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>E_Ox: edge of the window</t>
+        </is>
+      </c>
       <c r="M8" s="13" t="n">
         <v>0.0102634</v>
       </c>
@@ -1575,11 +1597,11 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>1.487</v>
+        <v>1.4</v>
       </c>
       <c r="G11" s="13" t="n"/>
       <c r="H11" s="13" t="n">
-        <v>-2.396</v>
+        <v>-2.4</v>
       </c>
       <c r="I11" s="13" t="n"/>
       <c r="J11" s="13" t="inlineStr">
@@ -1884,7 +1906,7 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>1.436</v>
+        <v>1.35</v>
       </c>
       <c r="G14" s="13" t="n"/>
       <c r="H14" s="13" t="n">
@@ -1990,8 +2012,14 @@
           <t>O=C1C=CC(N1C)=O</t>
         </is>
       </c>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13" t="n"/>
+      <c r="F15" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
       <c r="H15" s="13" t="n">
         <v>-0.95</v>
       </c>
@@ -2001,7 +2029,11 @@
           <t>https://doi.org/10.1016/S0040-4039(00)01248-X</t>
         </is>
       </c>
-      <c r="K15" s="13" t="n"/>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>E_Ox: edge of the window</t>
+        </is>
+      </c>
       <c r="M15" s="13" t="n">
         <v>0.0047896</v>
       </c>
@@ -2087,8 +2119,14 @@
           <t>CC(C(OCCCC)=O)=C</t>
         </is>
       </c>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="13" t="n"/>
+      <c r="F16" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
       <c r="H16" s="13" t="n">
         <v>-2.41</v>
       </c>
@@ -2098,7 +2136,11 @@
           <t>https://doi.org/10.1246/bcsj.51.339</t>
         </is>
       </c>
-      <c r="K16" s="13" t="n"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>E_Ox: edge of the window</t>
+        </is>
+      </c>
       <c r="M16" s="13" t="n">
         <v>0.00216672</v>
       </c>
@@ -2188,8 +2230,14 @@
         <v>1.72</v>
       </c>
       <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n"/>
+      <c r="H17" s="13" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>&lt;</t>
+        </is>
+      </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41929-023-01089-x</t>
@@ -2197,7 +2245,7 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>reduction potential not reported</t>
+          <t>E_Red: not reported; edge of the window</t>
         </is>
       </c>
       <c r="M17" s="13" t="n">
@@ -2299,14 +2347,10 @@
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="K18" s="13" t="inlineStr">
-        <is>
-          <t>measured by NHO/PAU; voltammogram not in the data</t>
-        </is>
-      </c>
+          <t>https://doi.org/10.1002/anie.9565676</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="n"/>
       <c r="M18" s="13" t="n">
         <v>0.00410537</v>
       </c>
@@ -2393,11 +2437,11 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>1.252</v>
+        <v>1.25</v>
       </c>
       <c r="G19" s="13" t="n"/>
       <c r="H19" s="13" t="n">
-        <v>-1.568</v>
+        <v>-1.6</v>
       </c>
       <c r="I19" s="13" t="n"/>
       <c r="J19" s="13" t="inlineStr">
@@ -2496,11 +2540,11 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.908</v>
+        <v>0.85</v>
       </c>
       <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n">
-        <v>-2.155</v>
+        <v>-2.15</v>
       </c>
       <c r="I20" s="13" t="n"/>
       <c r="J20" s="13" t="inlineStr">
@@ -2805,11 +2849,11 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>2.017</v>
+        <v>1.95</v>
       </c>
       <c r="G23" s="13" t="n"/>
       <c r="H23" s="13" t="n">
-        <v>-1.792</v>
+        <v>-1.8</v>
       </c>
       <c r="I23" s="13" t="n"/>
       <c r="J23" s="13" t="inlineStr">
@@ -2912,7 +2956,7 @@
       </c>
       <c r="G24" s="13" t="n"/>
       <c r="H24" s="13" t="n">
-        <v>-1.436</v>
+        <v>-1.4</v>
       </c>
       <c r="I24" s="13" t="n"/>
       <c r="J24" s="13" t="inlineStr">
@@ -3011,11 +3055,11 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>1.687</v>
+        <v>1.65</v>
       </c>
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n">
-        <v>-2.162</v>
+        <v>-2.15</v>
       </c>
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="13" t="inlineStr">
@@ -3114,11 +3158,11 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>1.895</v>
+        <v>1.85</v>
       </c>
       <c r="G26" s="13" t="n"/>
       <c r="H26" s="13" t="n">
-        <v>-2.318</v>
+        <v>-2.3</v>
       </c>
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="13" t="inlineStr">
@@ -3427,11 +3471,11 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>1.911</v>
+        <v>1.85</v>
       </c>
       <c r="G29" s="13" t="n"/>
       <c r="H29" s="13" t="n">
-        <v>-1.951</v>
+        <v>-1.95</v>
       </c>
       <c r="I29" s="13" t="n"/>
       <c r="J29" s="13" t="inlineStr">
@@ -3538,7 +3582,7 @@
         </is>
       </c>
       <c r="H30" s="13" t="n">
-        <v>-1.225</v>
+        <v>-1.15</v>
       </c>
       <c r="I30" s="13" t="n"/>
       <c r="J30" s="13" t="inlineStr">
@@ -3968,7 +4012,7 @@
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>estimated from Leandro's thioamides; no reference recorded</t>
+          <t>estimated from structurally related thioamides</t>
         </is>
       </c>
       <c r="M34" s="13" t="n">
@@ -4075,7 +4119,7 @@
       </c>
       <c r="K35" s="13" t="inlineStr">
         <is>
-          <t>estimated from Leandro's thioamides; no reference recorded</t>
+          <t>estimated from structurally related thioamides</t>
         </is>
       </c>
       <c r="M35" s="13" t="n">
@@ -4164,11 +4208,11 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>1.798</v>
+        <v>1.75</v>
       </c>
       <c r="G36" s="13" t="n"/>
       <c r="H36" s="13" t="n">
-        <v>-2.255</v>
+        <v>-2.25</v>
       </c>
       <c r="I36" s="13" t="n"/>
       <c r="J36" s="13" t="inlineStr">
@@ -4366,11 +4410,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>1.61</v>
+        <v>1.5</v>
       </c>
       <c r="G38" s="13" t="n"/>
       <c r="H38" s="13" t="n">
-        <v>-2.212</v>
+        <v>-2.3</v>
       </c>
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="inlineStr">
@@ -4469,11 +4513,11 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>1.93</v>
+        <v>1.9</v>
       </c>
       <c r="G39" s="13" t="n"/>
       <c r="H39" s="13" t="n">
-        <v>-2.288</v>
+        <v>-2.3</v>
       </c>
       <c r="I39" s="13" t="n"/>
       <c r="J39" s="13" t="inlineStr">
@@ -4679,11 +4723,11 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>1.675</v>
+        <v>1.6</v>
       </c>
       <c r="G41" s="13" t="n"/>
       <c r="H41" s="13" t="n">
-        <v>-2.1</v>
+        <v>-2</v>
       </c>
       <c r="I41" s="13" t="n"/>
       <c r="J41" s="13" t="inlineStr">
@@ -4980,11 +5024,11 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>2.189</v>
+        <v>2.2</v>
       </c>
       <c r="G44" s="13" t="n"/>
       <c r="H44" s="13" t="n">
-        <v>-1.6</v>
+        <v>-1.55</v>
       </c>
       <c r="I44" s="13" t="n"/>
       <c r="J44" s="13" t="inlineStr">
@@ -5083,11 +5127,11 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>2.017</v>
+        <v>1.95</v>
       </c>
       <c r="G45" s="13" t="n"/>
       <c r="H45" s="13" t="n">
-        <v>-1.698</v>
+        <v>-1.7</v>
       </c>
       <c r="I45" s="13" t="n"/>
       <c r="J45" s="13" t="inlineStr">
@@ -5194,7 +5238,7 @@
         </is>
       </c>
       <c r="H46" s="13" t="n">
-        <v>-1.736</v>
+        <v>-1.65</v>
       </c>
       <c r="I46" s="13" t="n"/>
       <c r="J46" s="13" t="inlineStr">
@@ -5396,11 +5440,11 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>1.884</v>
+        <v>1.55</v>
       </c>
       <c r="G48" s="13" t="n"/>
       <c r="H48" s="13" t="n">
-        <v>-2.291</v>
+        <v>-2.3</v>
       </c>
       <c r="I48" s="13" t="n"/>
       <c r="J48" s="13" t="inlineStr">
@@ -5498,8 +5542,14 @@
           <t>O=C(C1=CC=CC2=CC=CN=C21)OC</t>
         </is>
       </c>
-      <c r="F49" s="13" t="n"/>
-      <c r="G49" s="13" t="n"/>
+      <c r="F49" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
       <c r="H49" s="13" t="n">
         <v>-1.87</v>
       </c>
@@ -5509,7 +5559,11 @@
           <t>https://doi.org/10.1021/jacs.2c05687</t>
         </is>
       </c>
-      <c r="K49" s="13" t="n"/>
+      <c r="K49" s="13" t="inlineStr">
+        <is>
+          <t>E_Ox: edge of the window</t>
+        </is>
+      </c>
       <c r="M49" s="13" t="n">
         <v>0.0161934</v>
       </c>
@@ -5604,7 +5658,7 @@
         </is>
       </c>
       <c r="H50" s="13" t="n">
-        <v>-1.965</v>
+        <v>-2</v>
       </c>
       <c r="I50" s="13" t="n"/>
       <c r="J50" s="13" t="inlineStr">

</xml_diff>